<commit_message>
feat: imlement excel validation in src/core/validator.py; update main.py to integrate.
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -513,7 +513,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -559,7 +559,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement logs with src/core/logger.py; update main.py to integrate.
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: improve logs with metrics in src/main.py
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -538,7 +538,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: add latency, timeout and error simulation in src/sms/simulator.py; add retry in src/core/retry.py; update src/main.py to integrate
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,7 +492,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -584,14 +584,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>41278364750</v>
+        <v>4127836450</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -616,24 +616,45 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>2421536845</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>toplovo</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>gs-223</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
         <v>4227830099</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>gsm</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>it-443</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>ONLINE</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor: implement async parallelism; concurrency; internal queue management
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -538,7 +538,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>INOPERATIVO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>

</xml_diff>

<commit_message>
refactor: integrate one way execution server-main.py
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -471,10 +471,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ONLINE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>INOPERATIVO</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Dispositivo 4243742525 no respondió tras 3 intentos</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -492,10 +496,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ONLINE</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>INOPERATIVO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dispositivo 2448710098 no respondió tras 3 intentos</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -541,7 +549,11 @@
           <t>INOPERATIVO</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Dispositivo 4267386409 no respondió tras 3 intentos</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -584,10 +596,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ONLINE</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>INOPERATIVO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dispositivo 4127877894 no respondió tras 3 intentos</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -633,7 +649,11 @@
           <t>INOPERATIVO</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dispositivo 2421536845 no respondió tras 3 intentos</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -651,10 +671,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ONLINE</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>INOPERATIVO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Dispositivo 4227830099 no respondió tras 3 intentos</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add event logs for each ping from SMSgate in src/api/server.py
</commit_message>
<xml_diff>
--- a/data/localizadores.xlsx
+++ b/data/localizadores.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Toplovo</t>
+          <t>#Toplovo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -471,212 +471,237 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dispositivo 4243742525 no respondió tras 3 intentos</t>
+          <t>Marca no soportada: #toplovo</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2448710098</v>
+        <v>4243616194</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gsm</t>
+          <t>topfly</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>it-443</t>
+          <t>pionnerX 100</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>SIN_RESPUESTA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Dispositivo 2448710098 no respondió tras 3 intentos</t>
+          <t>No response</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4166718888</v>
+        <v>2448710098</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>perr</t>
+          <t>gsm</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>jhs10000</t>
+          <t>it-443</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NO SOPORTADO</t>
+          <t>SIN_RESPUESTA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Marca no soportada: perr</t>
+          <t>No response</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4267386409</v>
+        <v>4166718888</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>gsm</t>
+          <t>perr</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>fx-222</t>
+          <t>jhs10000</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dispositivo 4267386409 no respondió tras 3 intentos</t>
+          <t>Marca no soportada: perr</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4228769900</v>
+        <v>4267386409</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>frido</t>
+          <t>gsm</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>frd0010</t>
+          <t>fx-222</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NO SOPORTADO</t>
+          <t>SIN_RESPUESTA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Marca no soportada: frido</t>
+          <t>No response</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4127877894</v>
+        <v>4228769900</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>toplovo</t>
+          <t>frido</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>gs-223</t>
+          <t>frd0010</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Dispositivo 4127877894 no respondió tras 3 intentos</t>
+          <t>Marca no soportada: frido</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4127836450</v>
+        <v>4127877894</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gsm</t>
+          <t>toplovo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>it-9000</t>
+          <t>gs-223</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NO SOPORTADO</t>
+          <t>SIN_RESPUESTA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Modelo no soportado: gsm it-9000</t>
+          <t>No response</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2421536845</v>
+        <v>4127836450</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>toplovo</t>
+          <t>gsm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>gs-223</t>
+          <t>it-9000</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>INOPERATIVO</t>
+          <t>NO SOPORTADO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Dispositivo 2421536845 no respondió tras 3 intentos</t>
+          <t>Modelo no soportado: gsm it-9000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>2421536845</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>toplovo</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>gs-223</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SIN_RESPUESTA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No response</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>4227830099</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>gsm</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>it-443</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>INOPERATIVO</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Dispositivo 4227830099 no respondió tras 3 intentos</t>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SIN_RESPUESTA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No response</t>
         </is>
       </c>
     </row>

</xml_diff>